<commit_message>
graficas 2018 con el ancho que decide el programa
</commit_message>
<xml_diff>
--- a/Datos ESPARTACO/Parámetros para análisis de Antares/Resultados perfiles halpha 2018.xlsx
+++ b/Datos ESPARTACO/Parámetros para análisis de Antares/Resultados perfiles halpha 2018.xlsx
@@ -492,22 +492,22 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>6561.955</v>
+        <v>6562.019</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.000131</v>
+        <v>-0.000121</v>
       </c>
       <c r="F2" t="n">
-        <v>-39.1497</v>
+        <v>-36.2219</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2953</v>
+        <v>0.275</v>
       </c>
       <c r="H2" t="n">
-        <v>0.795</v>
+        <v>0.854</v>
       </c>
       <c r="I2" t="n">
-        <v>0.2518</v>
+        <v>0.2514</v>
       </c>
     </row>
     <row r="3">
@@ -527,22 +527,22 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>6563.048</v>
+        <v>6562.839</v>
       </c>
       <c r="E3" t="n">
-        <v>3.6e-05</v>
+        <v>4e-06</v>
       </c>
       <c r="F3" t="n">
-        <v>10.7707</v>
+        <v>1.2508</v>
       </c>
       <c r="G3" t="n">
-        <v>0.8426</v>
+        <v>0.8031</v>
       </c>
       <c r="H3" t="n">
-        <v>1.763</v>
+        <v>1.39</v>
       </c>
       <c r="I3" t="n">
-        <v>1.5929</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="4">
@@ -562,22 +562,22 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>6563.912</v>
+        <v>6563.812</v>
       </c>
       <c r="E4" t="n">
-        <v>7.8e-05</v>
+        <v>6.3e-05</v>
       </c>
       <c r="F4" t="n">
-        <v>23.5195</v>
+        <v>18.9484</v>
       </c>
       <c r="G4" t="n">
-        <v>0.1497</v>
+        <v>0.4258</v>
       </c>
       <c r="H4" t="n">
-        <v>0.607</v>
+        <v>1.014</v>
       </c>
       <c r="I4" t="n">
-        <v>0.1173</v>
+        <v>0.4842</v>
       </c>
     </row>
     <row r="5">
@@ -597,22 +597,22 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>6561.975</v>
+        <v>6562.148</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.000128</v>
+        <v>-0.000101</v>
       </c>
       <c r="F5" t="n">
-        <v>-38.2319</v>
+        <v>-30.3391</v>
       </c>
       <c r="G5" t="n">
-        <v>0.3526</v>
+        <v>0.1467</v>
       </c>
       <c r="H5" t="n">
-        <v>0.907</v>
+        <v>1.813</v>
       </c>
       <c r="I5" t="n">
-        <v>0.412</v>
+        <v>0.3827</v>
       </c>
     </row>
     <row r="6">
@@ -632,22 +632,22 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>6563.034</v>
+        <v>6562.733</v>
       </c>
       <c r="E6" t="n">
-        <v>3.4e-05</v>
+        <v>-1.2e-05</v>
       </c>
       <c r="F6" t="n">
-        <v>10.143</v>
+        <v>-3.5914</v>
       </c>
       <c r="G6" t="n">
-        <v>0.8673999999999999</v>
+        <v>0.6654</v>
       </c>
       <c r="H6" t="n">
-        <v>1.756</v>
+        <v>0.864</v>
       </c>
       <c r="I6" t="n">
-        <v>1.6414</v>
+        <v>0.62</v>
       </c>
     </row>
     <row r="7">
@@ -667,22 +667,22 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>6563.94</v>
+        <v>6563.578</v>
       </c>
       <c r="E7" t="n">
-        <v>8.3e-05</v>
+        <v>2.8e-05</v>
       </c>
       <c r="F7" t="n">
-        <v>24.7826</v>
+        <v>8.2697</v>
       </c>
       <c r="G7" t="n">
-        <v>0.1569</v>
+        <v>0.7365</v>
       </c>
       <c r="H7" t="n">
-        <v>0.607</v>
+        <v>1.222</v>
       </c>
       <c r="I7" t="n">
-        <v>0.1232</v>
+        <v>1.1079</v>
       </c>
     </row>
     <row r="8">
@@ -702,19 +702,19 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>6562.033</v>
+        <v>6562.11</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.000119</v>
+        <v>-0.000107</v>
       </c>
       <c r="F8" t="n">
-        <v>-35.5774</v>
+        <v>-32.0812</v>
       </c>
       <c r="G8" t="n">
-        <v>0.3703</v>
+        <v>0.3604</v>
       </c>
       <c r="H8" t="n">
-        <v>0.881</v>
+        <v>0.905</v>
       </c>
       <c r="I8" t="n">
         <v>0.3479</v>
@@ -737,22 +737,22 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>6563.047</v>
+        <v>6562.857</v>
       </c>
       <c r="E9" t="n">
-        <v>3.6e-05</v>
+        <v>7e-06</v>
       </c>
       <c r="F9" t="n">
-        <v>10.7183</v>
+        <v>2.073</v>
       </c>
       <c r="G9" t="n">
-        <v>0.8538</v>
+        <v>0.8391</v>
       </c>
       <c r="H9" t="n">
-        <v>1.794</v>
+        <v>1.426</v>
       </c>
       <c r="I9" t="n">
-        <v>1.6332</v>
+        <v>1.3018</v>
       </c>
     </row>
     <row r="10">
@@ -772,22 +772,22 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>6564.007</v>
+        <v>6563.9</v>
       </c>
       <c r="E10" t="n">
-        <v>9.3e-05</v>
+        <v>7.7e-05</v>
       </c>
       <c r="F10" t="n">
-        <v>27.8772</v>
+        <v>22.9622</v>
       </c>
       <c r="G10" t="n">
-        <v>0.2159</v>
+        <v>0.4535</v>
       </c>
       <c r="H10" t="n">
-        <v>0.607</v>
+        <v>0.994</v>
       </c>
       <c r="I10" t="n">
-        <v>0.1678</v>
+        <v>0.4978</v>
       </c>
     </row>
     <row r="11">
@@ -807,22 +807,22 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>6562.061</v>
+        <v>6562.178</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.000114</v>
+        <v>-9.7e-05</v>
       </c>
       <c r="F11" t="n">
-        <v>-34.2889</v>
+        <v>-28.9511</v>
       </c>
       <c r="G11" t="n">
-        <v>0.3313</v>
+        <v>0.3044</v>
       </c>
       <c r="H11" t="n">
-        <v>0.888</v>
+        <v>0.9389999999999999</v>
       </c>
       <c r="I11" t="n">
-        <v>0.3473</v>
+        <v>0.3463</v>
       </c>
     </row>
     <row r="12">
@@ -842,22 +842,22 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>6563.077</v>
+        <v>6562.863</v>
       </c>
       <c r="E12" t="n">
-        <v>4e-05</v>
+        <v>8e-06</v>
       </c>
       <c r="F12" t="n">
-        <v>12.1084</v>
+        <v>2.3299</v>
       </c>
       <c r="G12" t="n">
-        <v>0.8502999999999999</v>
+        <v>0.8246</v>
       </c>
       <c r="H12" t="n">
-        <v>1.684</v>
+        <v>1.256</v>
       </c>
       <c r="I12" t="n">
-        <v>1.546</v>
+        <v>1.1199</v>
       </c>
     </row>
     <row r="13">
@@ -877,22 +877,22 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>6563.961</v>
+        <v>6563.836</v>
       </c>
       <c r="E13" t="n">
-        <v>8.6e-05</v>
+        <v>6.7e-05</v>
       </c>
       <c r="F13" t="n">
-        <v>25.7618</v>
+        <v>20.0681</v>
       </c>
       <c r="G13" t="n">
-        <v>0.1967</v>
+        <v>0.5022</v>
       </c>
       <c r="H13" t="n">
-        <v>0.607</v>
+        <v>1</v>
       </c>
       <c r="I13" t="n">
-        <v>0.1549</v>
+        <v>0.5635</v>
       </c>
     </row>
     <row r="14">
@@ -912,22 +912,22 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>6562.047</v>
+        <v>6562.187</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.000117</v>
+        <v>-9.500000000000001e-05</v>
       </c>
       <c r="F14" t="n">
-        <v>-34.9354</v>
+        <v>-28.5319</v>
       </c>
       <c r="G14" t="n">
-        <v>0.3162</v>
+        <v>0.2023</v>
       </c>
       <c r="H14" t="n">
-        <v>0.884</v>
+        <v>1.05</v>
       </c>
       <c r="I14" t="n">
-        <v>0.3353</v>
+        <v>0.3223</v>
       </c>
     </row>
     <row r="15">
@@ -947,22 +947,22 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>6563.109</v>
+        <v>6562.853</v>
       </c>
       <c r="E15" t="n">
-        <v>4.5e-05</v>
+        <v>6e-06</v>
       </c>
       <c r="F15" t="n">
-        <v>13.55</v>
+        <v>1.8728</v>
       </c>
       <c r="G15" t="n">
-        <v>0.8391999999999999</v>
+        <v>0.7468</v>
       </c>
       <c r="H15" t="n">
-        <v>1.683</v>
+        <v>1.036</v>
       </c>
       <c r="I15" t="n">
-        <v>1.5372</v>
+        <v>0.8446</v>
       </c>
     </row>
     <row r="16">
@@ -982,22 +982,22 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>6564.003</v>
+        <v>6563.764</v>
       </c>
       <c r="E16" t="n">
-        <v>9.2e-05</v>
+        <v>5.6e-05</v>
       </c>
       <c r="F16" t="n">
-        <v>27.6636</v>
+        <v>16.7692</v>
       </c>
       <c r="G16" t="n">
-        <v>0.1927</v>
+        <v>0.6206</v>
       </c>
       <c r="H16" t="n">
-        <v>0.607</v>
+        <v>1.096</v>
       </c>
       <c r="I16" t="n">
-        <v>0.1529</v>
+        <v>0.8090000000000001</v>
       </c>
     </row>
     <row r="17">
@@ -1017,22 +1017,22 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>6562.064</v>
+        <v>6562.167</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.000114</v>
+        <v>-9.8e-05</v>
       </c>
       <c r="F17" t="n">
-        <v>-34.1532</v>
+        <v>-29.4756</v>
       </c>
       <c r="G17" t="n">
-        <v>0.268</v>
+        <v>0.1733</v>
       </c>
       <c r="H17" t="n">
-        <v>0.855</v>
+        <v>0.95</v>
       </c>
       <c r="I17" t="n">
-        <v>0.2603</v>
+        <v>0.2505</v>
       </c>
     </row>
     <row r="18">
@@ -1052,22 +1052,22 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>6563.146</v>
+        <v>6562.935</v>
       </c>
       <c r="E18" t="n">
-        <v>5.1e-05</v>
+        <v>1.9e-05</v>
       </c>
       <c r="F18" t="n">
-        <v>15.2679</v>
+        <v>5.6169</v>
       </c>
       <c r="G18" t="n">
-        <v>0.8252</v>
+        <v>0.7798</v>
       </c>
       <c r="H18" t="n">
-        <v>1.62</v>
+        <v>1.088</v>
       </c>
       <c r="I18" t="n">
-        <v>1.4484</v>
+        <v>0.9237</v>
       </c>
     </row>
     <row r="19">
@@ -1087,22 +1087,22 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>6564.006</v>
+        <v>6563.847</v>
       </c>
       <c r="E19" t="n">
-        <v>9.3e-05</v>
+        <v>6.9e-05</v>
       </c>
       <c r="F19" t="n">
-        <v>27.8341</v>
+        <v>20.5586</v>
       </c>
       <c r="G19" t="n">
-        <v>0.2012</v>
+        <v>0.5595</v>
       </c>
       <c r="H19" t="n">
-        <v>0.607</v>
+        <v>0.988</v>
       </c>
       <c r="I19" t="n">
-        <v>0.1589</v>
+        <v>0.6206</v>
       </c>
     </row>
     <row r="20">
@@ -1122,22 +1122,22 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>6562.083</v>
+        <v>6562.028</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.000111</v>
+        <v>-0.000119</v>
       </c>
       <c r="F20" t="n">
-        <v>-33.3053</v>
+        <v>-35.822</v>
       </c>
       <c r="G20" t="n">
-        <v>0.2973</v>
+        <v>0.1309</v>
       </c>
       <c r="H20" t="n">
         <v>0.909</v>
       </c>
       <c r="I20" t="n">
-        <v>0.2916</v>
+        <v>0.1282</v>
       </c>
     </row>
     <row r="21">
@@ -1157,22 +1157,22 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>6563.186</v>
+        <v>6562.962</v>
       </c>
       <c r="E21" t="n">
-        <v>5.7e-05</v>
+        <v>2.3e-05</v>
       </c>
       <c r="F21" t="n">
-        <v>17.1064</v>
+        <v>6.8321</v>
       </c>
       <c r="G21" t="n">
-        <v>0.8129999999999999</v>
+        <v>0.6758999999999999</v>
       </c>
       <c r="H21" t="n">
-        <v>1.732</v>
+        <v>1.029</v>
       </c>
       <c r="I21" t="n">
-        <v>1.5193</v>
+        <v>0.7495000000000001</v>
       </c>
     </row>
     <row r="22">
@@ -1192,22 +1192,22 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>6564.029</v>
+        <v>6563.838</v>
       </c>
       <c r="E22" t="n">
-        <v>9.6e-05</v>
+        <v>6.7e-05</v>
       </c>
       <c r="F22" t="n">
-        <v>28.8849</v>
+        <v>20.1289</v>
       </c>
       <c r="G22" t="n">
-        <v>0.1563</v>
+        <v>0.5826</v>
       </c>
       <c r="H22" t="n">
-        <v>0.607</v>
+        <v>1.092</v>
       </c>
       <c r="I22" t="n">
-        <v>0.123</v>
+        <v>0.746</v>
       </c>
     </row>
     <row r="23">
@@ -1227,22 +1227,22 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>6562.111</v>
+        <v>6562.203</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.000107</v>
+        <v>-9.3e-05</v>
       </c>
       <c r="F23" t="n">
-        <v>-32.0015</v>
+        <v>-27.8268</v>
       </c>
       <c r="G23" t="n">
-        <v>0.3545</v>
+        <v>0.2286</v>
       </c>
       <c r="H23" t="n">
-        <v>0.924</v>
+        <v>1.123</v>
       </c>
       <c r="I23" t="n">
-        <v>0.4002</v>
+        <v>0.3859</v>
       </c>
     </row>
     <row r="24">
@@ -1262,22 +1262,22 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>6563.141</v>
+        <v>6562.893</v>
       </c>
       <c r="E24" t="n">
-        <v>5e-05</v>
+        <v>1.2e-05</v>
       </c>
       <c r="F24" t="n">
-        <v>15.0405</v>
+        <v>3.7157</v>
       </c>
       <c r="G24" t="n">
-        <v>0.8458</v>
+        <v>0.7415</v>
       </c>
       <c r="H24" t="n">
-        <v>1.726</v>
+        <v>1.03</v>
       </c>
       <c r="I24" t="n">
-        <v>1.5838</v>
+        <v>0.9076</v>
       </c>
     </row>
     <row r="25">
@@ -1297,22 +1297,22 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>6564.032</v>
+        <v>6563.782</v>
       </c>
       <c r="E25" t="n">
-        <v>9.7e-05</v>
+        <v>5.9e-05</v>
       </c>
       <c r="F25" t="n">
-        <v>29.0254</v>
+        <v>17.5784</v>
       </c>
       <c r="G25" t="n">
-        <v>0.177</v>
+        <v>0.6052</v>
       </c>
       <c r="H25" t="n">
-        <v>0.607</v>
+        <v>1.123</v>
       </c>
       <c r="I25" t="n">
-        <v>0.1394</v>
+        <v>0.8089</v>
       </c>
     </row>
     <row r="26">
@@ -1332,22 +1332,22 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>6562.079</v>
+        <v>6562.256</v>
       </c>
       <c r="E26" t="n">
-        <v>-0.000112</v>
+        <v>-8.500000000000001e-05</v>
       </c>
       <c r="F26" t="n">
-        <v>-33.4914</v>
+        <v>-25.4051</v>
       </c>
       <c r="G26" t="n">
-        <v>0.2732</v>
+        <v>0.2248</v>
       </c>
       <c r="H26" t="n">
-        <v>0.864</v>
+        <v>1</v>
       </c>
       <c r="I26" t="n">
-        <v>0.254</v>
+        <v>0.2523</v>
       </c>
     </row>
     <row r="27">
@@ -1367,22 +1367,22 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>6563.207</v>
+        <v>6562.909</v>
       </c>
       <c r="E27" t="n">
-        <v>6e-05</v>
+        <v>1.5e-05</v>
       </c>
       <c r="F27" t="n">
-        <v>18.0426</v>
+        <v>4.4477</v>
       </c>
       <c r="G27" t="n">
-        <v>0.8495</v>
+        <v>0.7773</v>
       </c>
       <c r="H27" t="n">
-        <v>1.742</v>
+        <v>1.157</v>
       </c>
       <c r="I27" t="n">
-        <v>1.5926</v>
+        <v>0.9671</v>
       </c>
     </row>
     <row r="28">
@@ -1402,22 +1402,22 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>6564.084</v>
+        <v>6563.873</v>
       </c>
       <c r="E28" t="n">
-        <v>0.000105</v>
+        <v>7.2e-05</v>
       </c>
       <c r="F28" t="n">
-        <v>31.3822</v>
+        <v>21.7327</v>
       </c>
       <c r="G28" t="n">
-        <v>0.1474</v>
+        <v>0.5713</v>
       </c>
       <c r="H28" t="n">
-        <v>0.607</v>
+        <v>1.117</v>
       </c>
       <c r="I28" t="n">
-        <v>0.116</v>
+        <v>0.7573</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Arreglo de la profundidad y el ancho de los espectros
</commit_message>
<xml_diff>
--- a/Datos ESPARTACO/Parámetros para análisis de Antares/Resultados perfiles halpha 2018.xlsx
+++ b/Datos ESPARTACO/Parámetros para análisis de Antares/Resultados perfiles halpha 2018.xlsx
@@ -483,7 +483,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>halpha</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -492,22 +492,22 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>6562.019</v>
+        <v>6561.937</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.000121</v>
+        <v>-0.000133</v>
       </c>
       <c r="F2" t="n">
-        <v>-36.2219</v>
+        <v>-39.9867</v>
       </c>
       <c r="G2" t="n">
-        <v>0.275</v>
+        <v>0.1179</v>
       </c>
       <c r="H2" t="n">
-        <v>0.854</v>
+        <v>0.716</v>
       </c>
       <c r="I2" t="n">
-        <v>0.2514</v>
+        <v>0.0905</v>
       </c>
     </row>
     <row r="3">
@@ -518,7 +518,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>halpha</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -527,22 +527,22 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>6562.839</v>
+        <v>6562.874</v>
       </c>
       <c r="E3" t="n">
-        <v>4e-06</v>
+        <v>9e-06</v>
       </c>
       <c r="F3" t="n">
-        <v>1.2508</v>
+        <v>2.8147</v>
       </c>
       <c r="G3" t="n">
-        <v>0.8031</v>
+        <v>0.7847</v>
       </c>
       <c r="H3" t="n">
-        <v>1.39</v>
+        <v>1.092</v>
       </c>
       <c r="I3" t="n">
-        <v>1.25</v>
+        <v>0.9183</v>
       </c>
     </row>
     <row r="4">
@@ -553,7 +553,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>halpha</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -562,22 +562,22 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>6563.812</v>
+        <v>6563.806</v>
       </c>
       <c r="E4" t="n">
-        <v>6.3e-05</v>
+        <v>6.2e-05</v>
       </c>
       <c r="F4" t="n">
-        <v>18.9484</v>
+        <v>18.7</v>
       </c>
       <c r="G4" t="n">
-        <v>0.4258</v>
+        <v>0.5631</v>
       </c>
       <c r="H4" t="n">
-        <v>1.014</v>
+        <v>0.967</v>
       </c>
       <c r="I4" t="n">
-        <v>0.4842</v>
+        <v>0.6405999999999999</v>
       </c>
     </row>
     <row r="5">
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>halpha</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -597,22 +597,22 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>6562.148</v>
+        <v>6560.974</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.000101</v>
+        <v>-0.00028</v>
       </c>
       <c r="F5" t="n">
-        <v>-30.3391</v>
+        <v>-83.96250000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1467</v>
+        <v>0.07770000000000001</v>
       </c>
       <c r="H5" t="n">
-        <v>1.813</v>
+        <v>4.044</v>
       </c>
       <c r="I5" t="n">
-        <v>0.3827</v>
+        <v>0.3686</v>
       </c>
     </row>
     <row r="6">
@@ -623,7 +623,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>halpha</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -632,22 +632,22 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>6562.733</v>
+        <v>6562.914</v>
       </c>
       <c r="E6" t="n">
-        <v>-1.2e-05</v>
+        <v>1.5e-05</v>
       </c>
       <c r="F6" t="n">
-        <v>-3.5914</v>
+        <v>4.6448</v>
       </c>
       <c r="G6" t="n">
-        <v>0.6654</v>
+        <v>0.8252</v>
       </c>
       <c r="H6" t="n">
-        <v>0.864</v>
+        <v>1.012</v>
       </c>
       <c r="I6" t="n">
-        <v>0.62</v>
+        <v>0.9162</v>
       </c>
     </row>
     <row r="7">
@@ -658,7 +658,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>halpha</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -667,22 +667,22 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>6563.578</v>
+        <v>6563.822</v>
       </c>
       <c r="E7" t="n">
-        <v>2.8e-05</v>
+        <v>6.499999999999999e-05</v>
       </c>
       <c r="F7" t="n">
-        <v>8.2697</v>
+        <v>19.4</v>
       </c>
       <c r="G7" t="n">
-        <v>0.7365</v>
+        <v>0.5504</v>
       </c>
       <c r="H7" t="n">
-        <v>1.222</v>
+        <v>0.959</v>
       </c>
       <c r="I7" t="n">
-        <v>1.1079</v>
+        <v>0.6089</v>
       </c>
     </row>
     <row r="8">
@@ -693,7 +693,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>sector_naranja</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -702,22 +702,22 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>6562.11</v>
+        <v>6562.008</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.000107</v>
+        <v>-0.000122</v>
       </c>
       <c r="F8" t="n">
-        <v>-32.0812</v>
+        <v>-36.7212</v>
       </c>
       <c r="G8" t="n">
-        <v>0.3604</v>
+        <v>0.1475</v>
       </c>
       <c r="H8" t="n">
-        <v>0.905</v>
+        <v>0.766</v>
       </c>
       <c r="I8" t="n">
-        <v>0.3479</v>
+        <v>0.1235</v>
       </c>
     </row>
     <row r="9">
@@ -728,7 +728,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>sector_naranja</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -737,22 +737,22 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>6562.857</v>
+        <v>6562.948</v>
       </c>
       <c r="E9" t="n">
-        <v>7e-06</v>
+        <v>2.1e-05</v>
       </c>
       <c r="F9" t="n">
-        <v>2.073</v>
+        <v>6.2216</v>
       </c>
       <c r="G9" t="n">
-        <v>0.8391</v>
+        <v>0.8139999999999999</v>
       </c>
       <c r="H9" t="n">
-        <v>1.426</v>
+        <v>1.118</v>
       </c>
       <c r="I9" t="n">
-        <v>1.3018</v>
+        <v>0.9757</v>
       </c>
     </row>
     <row r="10">
@@ -763,7 +763,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>sector_naranja</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -772,22 +772,22 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>6563.9</v>
+        <v>6563.911</v>
       </c>
       <c r="E10" t="n">
-        <v>7.7e-05</v>
+        <v>7.8e-05</v>
       </c>
       <c r="F10" t="n">
-        <v>22.9622</v>
+        <v>23.4701</v>
       </c>
       <c r="G10" t="n">
-        <v>0.4535</v>
+        <v>0.5656</v>
       </c>
       <c r="H10" t="n">
-        <v>0.994</v>
+        <v>0.927</v>
       </c>
       <c r="I10" t="n">
-        <v>0.4978</v>
+        <v>0.5998</v>
       </c>
     </row>
     <row r="11">
@@ -798,7 +798,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>halpha</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -807,22 +807,22 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>6562.178</v>
+        <v>6562.243</v>
       </c>
       <c r="E11" t="n">
-        <v>-9.7e-05</v>
+        <v>-8.7e-05</v>
       </c>
       <c r="F11" t="n">
-        <v>-28.9511</v>
+        <v>-26.0129</v>
       </c>
       <c r="G11" t="n">
-        <v>0.3044</v>
+        <v>0.1752</v>
       </c>
       <c r="H11" t="n">
-        <v>0.9389999999999999</v>
+        <v>1.262</v>
       </c>
       <c r="I11" t="n">
-        <v>0.3463</v>
+        <v>0.3308</v>
       </c>
     </row>
     <row r="12">
@@ -833,7 +833,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>halpha</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -842,22 +842,22 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>6562.863</v>
+        <v>6562.949</v>
       </c>
       <c r="E12" t="n">
-        <v>8e-06</v>
+        <v>2.1e-05</v>
       </c>
       <c r="F12" t="n">
-        <v>2.3299</v>
+        <v>6.2385</v>
       </c>
       <c r="G12" t="n">
-        <v>0.8246</v>
+        <v>0.8877</v>
       </c>
       <c r="H12" t="n">
-        <v>1.256</v>
+        <v>1.109</v>
       </c>
       <c r="I12" t="n">
-        <v>1.1199</v>
+        <v>1.0698</v>
       </c>
     </row>
     <row r="13">
@@ -868,7 +868,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>halpha</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -877,22 +877,22 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>6563.836</v>
+        <v>6563.909</v>
       </c>
       <c r="E13" t="n">
-        <v>6.7e-05</v>
+        <v>7.8e-05</v>
       </c>
       <c r="F13" t="n">
-        <v>20.0681</v>
+        <v>23.4</v>
       </c>
       <c r="G13" t="n">
-        <v>0.5022</v>
+        <v>0.5557</v>
       </c>
       <c r="H13" t="n">
-        <v>1</v>
+        <v>0.881</v>
       </c>
       <c r="I13" t="n">
-        <v>0.5635</v>
+        <v>0.5569</v>
       </c>
     </row>
     <row r="14">
@@ -903,7 +903,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>halpha</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -912,22 +912,22 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>6562.187</v>
+        <v>6562.165</v>
       </c>
       <c r="E14" t="n">
-        <v>-9.500000000000001e-05</v>
+        <v>-9.899999999999999e-05</v>
       </c>
       <c r="F14" t="n">
-        <v>-28.5319</v>
+        <v>-29.5569</v>
       </c>
       <c r="G14" t="n">
-        <v>0.2023</v>
+        <v>0.1769</v>
       </c>
       <c r="H14" t="n">
-        <v>1.05</v>
+        <v>1.199</v>
       </c>
       <c r="I14" t="n">
-        <v>0.3223</v>
+        <v>0.3199</v>
       </c>
     </row>
     <row r="15">
@@ -938,7 +938,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>halpha</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -947,22 +947,22 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>6562.853</v>
+        <v>6562.964</v>
       </c>
       <c r="E15" t="n">
-        <v>6e-06</v>
+        <v>2.3e-05</v>
       </c>
       <c r="F15" t="n">
-        <v>1.8728</v>
+        <v>6.9449</v>
       </c>
       <c r="G15" t="n">
-        <v>0.7468</v>
+        <v>0.8496</v>
       </c>
       <c r="H15" t="n">
-        <v>1.036</v>
+        <v>1.124</v>
       </c>
       <c r="I15" t="n">
-        <v>0.8446</v>
+        <v>1.0421</v>
       </c>
     </row>
     <row r="16">
@@ -973,7 +973,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>halpha</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -982,22 +982,22 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>6563.764</v>
+        <v>6563.927</v>
       </c>
       <c r="E16" t="n">
-        <v>5.6e-05</v>
+        <v>8.1e-05</v>
       </c>
       <c r="F16" t="n">
-        <v>16.7692</v>
+        <v>24.2</v>
       </c>
       <c r="G16" t="n">
-        <v>0.6206</v>
+        <v>0.5531</v>
       </c>
       <c r="H16" t="n">
-        <v>1.096</v>
+        <v>0.887</v>
       </c>
       <c r="I16" t="n">
-        <v>0.8090000000000001</v>
+        <v>0.6073</v>
       </c>
     </row>
     <row r="17">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>halpha</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1017,22 +1017,22 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>6562.167</v>
+        <v>6562.155</v>
       </c>
       <c r="E17" t="n">
-        <v>-9.8e-05</v>
+        <v>-0.0001</v>
       </c>
       <c r="F17" t="n">
-        <v>-29.4756</v>
+        <v>-29.9947</v>
       </c>
       <c r="G17" t="n">
-        <v>0.1733</v>
+        <v>0.1388</v>
       </c>
       <c r="H17" t="n">
-        <v>0.95</v>
+        <v>1.184</v>
       </c>
       <c r="I17" t="n">
-        <v>0.2505</v>
+        <v>0.2473</v>
       </c>
     </row>
     <row r="18">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>halpha</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1052,22 +1052,22 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>6562.935</v>
+        <v>6562.994</v>
       </c>
       <c r="E18" t="n">
-        <v>1.9e-05</v>
+        <v>2.8e-05</v>
       </c>
       <c r="F18" t="n">
-        <v>5.6169</v>
+        <v>8.299799999999999</v>
       </c>
       <c r="G18" t="n">
-        <v>0.7798</v>
+        <v>0.8408</v>
       </c>
       <c r="H18" t="n">
-        <v>1.088</v>
+        <v>1.089</v>
       </c>
       <c r="I18" t="n">
-        <v>0.9237</v>
+        <v>0.997</v>
       </c>
     </row>
     <row r="19">
@@ -1078,7 +1078,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>halpha</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1087,22 +1087,22 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>6563.847</v>
+        <v>6563.938</v>
       </c>
       <c r="E19" t="n">
-        <v>6.9e-05</v>
+        <v>8.2e-05</v>
       </c>
       <c r="F19" t="n">
-        <v>20.5586</v>
+        <v>24.7</v>
       </c>
       <c r="G19" t="n">
-        <v>0.5595</v>
+        <v>0.5545</v>
       </c>
       <c r="H19" t="n">
-        <v>0.988</v>
+        <v>0.875</v>
       </c>
       <c r="I19" t="n">
-        <v>0.6206</v>
+        <v>0.5531</v>
       </c>
     </row>
     <row r="20">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>halpha</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1122,22 +1122,22 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>6562.028</v>
+        <v>6561.929</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.000119</v>
+        <v>-0.000134</v>
       </c>
       <c r="F20" t="n">
-        <v>-35.822</v>
+        <v>-40.3177</v>
       </c>
       <c r="G20" t="n">
-        <v>0.1309</v>
+        <v>0.1143</v>
       </c>
       <c r="H20" t="n">
-        <v>0.909</v>
+        <v>0.768</v>
       </c>
       <c r="I20" t="n">
-        <v>0.1282</v>
+        <v>0.09859999999999999</v>
       </c>
     </row>
     <row r="21">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>halpha</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1157,22 +1157,22 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>6562.962</v>
+        <v>6563.05</v>
       </c>
       <c r="E21" t="n">
-        <v>2.3e-05</v>
+        <v>3.6e-05</v>
       </c>
       <c r="F21" t="n">
-        <v>6.8321</v>
+        <v>10.8545</v>
       </c>
       <c r="G21" t="n">
-        <v>0.6758999999999999</v>
+        <v>0.7625</v>
       </c>
       <c r="H21" t="n">
-        <v>1.029</v>
+        <v>1.04</v>
       </c>
       <c r="I21" t="n">
-        <v>0.7495000000000001</v>
+        <v>0.8535</v>
       </c>
     </row>
     <row r="22">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>halpha</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1192,22 +1192,22 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>6563.838</v>
+        <v>6563.955</v>
       </c>
       <c r="E22" t="n">
-        <v>6.7e-05</v>
+        <v>8.500000000000001e-05</v>
       </c>
       <c r="F22" t="n">
-        <v>20.1289</v>
+        <v>25.5</v>
       </c>
       <c r="G22" t="n">
-        <v>0.5826</v>
+        <v>0.5606</v>
       </c>
       <c r="H22" t="n">
-        <v>1.092</v>
+        <v>0.911</v>
       </c>
       <c r="I22" t="n">
-        <v>0.746</v>
+        <v>0.6274</v>
       </c>
     </row>
     <row r="23">
@@ -1218,7 +1218,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>halpha</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1227,22 +1227,22 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>6562.203</v>
+        <v>6562.177</v>
       </c>
       <c r="E23" t="n">
-        <v>-9.3e-05</v>
+        <v>-9.7e-05</v>
       </c>
       <c r="F23" t="n">
-        <v>-27.8268</v>
+        <v>-28.9943</v>
       </c>
       <c r="G23" t="n">
-        <v>0.2286</v>
+        <v>0.1724</v>
       </c>
       <c r="H23" t="n">
-        <v>1.123</v>
+        <v>1.082</v>
       </c>
       <c r="I23" t="n">
-        <v>0.3859</v>
+        <v>0.2813</v>
       </c>
     </row>
     <row r="24">
@@ -1253,7 +1253,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>halpha</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1262,22 +1262,22 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>6562.893</v>
+        <v>6563.011</v>
       </c>
       <c r="E24" t="n">
-        <v>1.2e-05</v>
+        <v>3e-05</v>
       </c>
       <c r="F24" t="n">
-        <v>3.7157</v>
+        <v>9.110900000000001</v>
       </c>
       <c r="G24" t="n">
-        <v>0.7415</v>
+        <v>0.8294</v>
       </c>
       <c r="H24" t="n">
-        <v>1.03</v>
+        <v>1.092</v>
       </c>
       <c r="I24" t="n">
-        <v>0.9076</v>
+        <v>0.9762999999999999</v>
       </c>
     </row>
     <row r="25">
@@ -1288,7 +1288,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>halpha</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1297,22 +1297,22 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>6563.782</v>
+        <v>6563.964</v>
       </c>
       <c r="E25" t="n">
-        <v>5.9e-05</v>
+        <v>8.6e-05</v>
       </c>
       <c r="F25" t="n">
-        <v>17.5784</v>
+        <v>25.9</v>
       </c>
       <c r="G25" t="n">
-        <v>0.6052</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="H25" t="n">
-        <v>1.123</v>
+        <v>0.906</v>
       </c>
       <c r="I25" t="n">
-        <v>0.8089</v>
+        <v>0.6207</v>
       </c>
     </row>
     <row r="26">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>halpha</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1332,22 +1332,22 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>6562.256</v>
+        <v>6562.04</v>
       </c>
       <c r="E26" t="n">
-        <v>-8.500000000000001e-05</v>
+        <v>-0.000118</v>
       </c>
       <c r="F26" t="n">
-        <v>-25.4051</v>
+        <v>-35.2507</v>
       </c>
       <c r="G26" t="n">
-        <v>0.2248</v>
+        <v>0.1089</v>
       </c>
       <c r="H26" t="n">
-        <v>1</v>
+        <v>0.897</v>
       </c>
       <c r="I26" t="n">
-        <v>0.2523</v>
+        <v>0.1056</v>
       </c>
     </row>
     <row r="27">
@@ -1358,7 +1358,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>halpha</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1367,22 +1367,22 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>6562.909</v>
+        <v>6563.018</v>
       </c>
       <c r="E27" t="n">
-        <v>1.5e-05</v>
+        <v>3.1e-05</v>
       </c>
       <c r="F27" t="n">
-        <v>4.4477</v>
+        <v>9.4283</v>
       </c>
       <c r="G27" t="n">
-        <v>0.7773</v>
+        <v>0.7852</v>
       </c>
       <c r="H27" t="n">
-        <v>1.157</v>
+        <v>1.086</v>
       </c>
       <c r="I27" t="n">
-        <v>0.9671</v>
+        <v>0.9171</v>
       </c>
     </row>
     <row r="28">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>libre</t>
+          <t>halpha</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1402,22 +1402,22 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>6563.873</v>
+        <v>6563.955</v>
       </c>
       <c r="E28" t="n">
-        <v>7.2e-05</v>
+        <v>8.500000000000001e-05</v>
       </c>
       <c r="F28" t="n">
-        <v>21.7327</v>
+        <v>25.5</v>
       </c>
       <c r="G28" t="n">
-        <v>0.5713</v>
+        <v>0.5614</v>
       </c>
       <c r="H28" t="n">
-        <v>1.117</v>
+        <v>1</v>
       </c>
       <c r="I28" t="n">
-        <v>0.7573</v>
+        <v>0.6652</v>
       </c>
     </row>
   </sheetData>

</xml_diff>